<commit_message>
Stage 5 Wave 3: mint people rows for reverse-orphan profiles (applied to prod 2026-07-19) + tracker: add open watch items
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-07-10.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-07-10.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="13" min="1" max="1"/>
@@ -4486,8 +4486,235 @@
         </is>
       </c>
     </row>
+    <row r="163" ht="21.75" customHeight="1" s="14">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
+        </is>
+      </c>
+      <c r="B163" s="17" t="n"/>
+      <c r="C163" s="17" t="n"/>
+      <c r="D163" s="17" t="n"/>
+      <c r="E163" s="18" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="19" t="inlineStr">
+        <is>
+          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
+        </is>
+      </c>
+      <c r="B164" s="26" t="inlineStr">
+        <is>
+          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
+        </is>
+      </c>
+      <c r="C164" s="26" t="inlineStr">
+        <is>
+          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
+        </is>
+      </c>
+      <c r="D164" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E164" s="26" t="inlineStr">
+        <is>
+          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="19" t="inlineStr">
+        <is>
+          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
+        </is>
+      </c>
+      <c r="B165" s="26" t="inlineStr">
+        <is>
+          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
+        </is>
+      </c>
+      <c r="C165" s="26" t="inlineStr">
+        <is>
+          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
+        </is>
+      </c>
+      <c r="D165" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E165" s="26" t="inlineStr">
+        <is>
+          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="19" t="inlineStr">
+        <is>
+          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
+        </is>
+      </c>
+      <c r="B166" s="26" t="inlineStr">
+        <is>
+          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
+        </is>
+      </c>
+      <c r="C166" s="26" t="inlineStr">
+        <is>
+          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
+        </is>
+      </c>
+      <c r="D166" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E166" s="26" t="inlineStr">
+        <is>
+          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="19" t="inlineStr">
+        <is>
+          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
+        </is>
+      </c>
+      <c r="B167" s="26" t="inlineStr">
+        <is>
+          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
+        </is>
+      </c>
+      <c r="C167" s="26" t="inlineStr">
+        <is>
+          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
+        </is>
+      </c>
+      <c r="D167" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E167" s="26" t="inlineStr">
+        <is>
+          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="19" t="inlineStr">
+        <is>
+          <t>Delete the stray Stripe Connect account</t>
+        </is>
+      </c>
+      <c r="B168" s="26" t="inlineStr">
+        <is>
+          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
+        </is>
+      </c>
+      <c r="C168" s="26" t="inlineStr">
+        <is>
+          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
+        </is>
+      </c>
+      <c r="D168" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E168" s="26" t="inlineStr">
+        <is>
+          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="19" t="inlineStr">
+        <is>
+          <t>ManyChat - disconnect the Instagram-side integration</t>
+        </is>
+      </c>
+      <c r="B169" s="26" t="inlineStr">
+        <is>
+          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+        </is>
+      </c>
+      <c r="C169" s="26" t="inlineStr">
+        <is>
+          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+        </is>
+      </c>
+      <c r="D169" s="21" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E169" s="26" t="inlineStr">
+        <is>
+          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="19" t="inlineStr">
+        <is>
+          <t>DB / Stripe drift watch items</t>
+        </is>
+      </c>
+      <c r="B170" s="26" t="inlineStr">
+        <is>
+          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+        </is>
+      </c>
+      <c r="C170" s="26" t="inlineStr">
+        <is>
+          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+        </is>
+      </c>
+      <c r="D170" s="21" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="E170" s="26" t="inlineStr">
+        <is>
+          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="19" t="inlineStr">
+        <is>
+          <t>Waitlist claim links - monitor first real-world use</t>
+        </is>
+      </c>
+      <c r="B171" s="26" t="inlineStr">
+        <is>
+          <t>Cancel frees a seat -&gt; the first waitlister is emailed a 24h claim link -&gt; they claim it. Rehearsed as a full matrix on develop and shipped to prod; needs a read-only confirm on its first genuine use.</t>
+        </is>
+      </c>
+      <c r="C171" s="26" t="inlineStr">
+        <is>
+          <t>On the next real cancellation that frees a seat on a full, waitlisted event, confirm: notified_at/expires_at stamped, the email sent, the claimant claimed (member_rsvp with metadata source=waitlist_claim), and the waitlist row deleted.</t>
+        </is>
+      </c>
+      <c r="D171" s="21" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E171" s="26" t="inlineStr">
+        <is>
+          <t>Shipped 2026-07-19. Zero-cost proof on first real use, like the Remove &amp; Refund WAIT-mode row.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A60:E60"/>
@@ -4500,6 +4727,7 @@
     <mergeCell ref="A74:E74"/>
     <mergeCell ref="A105:E105"/>
     <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A163:E163"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>

</xml_diff>